<commit_message>
Switch disposition vocabulary to five terms: retain, invest, consolidate, replace, retire
Bina Din changed the Step 4 output vocabulary on 2026-08-14, superseding her
2026-08-13 four-term decision. Under the old vocabulary `invest` covered both a
healthy application left alone and one carrying a funded remediation, separated
only by priority; `retain` is now its own disposition, so `invest` always means a
deliberate injection of money or effort.

Updated REQ 4, 27, 52 and 64 plus the Notes & assumptions and README statements
of the decision. In REQ 52's lookup table the all-pass key PPPP moves from
invest (Very Low) to retain (Very Low); every remaining invest row fails at least
one gate. Requirement count unchanged at 65. Also recorded Bina's four other
answers of the same date on risk substitution, cost's role in disposition, the
value dimension weighting, and the modelled cost-efficiency peer band.
</commit_message>
<xml_diff>
--- a/docs/requirements/Application Rationalization Agent Requirements - filled.xlsx
+++ b/docs/requirements/Application Rationalization Agent Requirements - filled.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overarching Prompt" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; assumptions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Overarching Prompt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes &amp; assumptions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -580,7 +580,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Analyze collected data and categorize applications into four separate categories (invest, consolidate, replace, or retire) based on critical data points.</t>
+          <t>Analyze collected data and categorize applications into five separate categories (retain, invest, consolidate, replace, or retire) based on critical data points.</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>(Step 4) Extend REQ 4: assign every application a disposition from exactly four categories - invest, consolidate, replace, retire - using the pass/fail gate engine specified in REQ 52 rather than a business-value-by-technical-health 2x2 (a 2x2 has no axis on which 'consolidate' can appear, and consolidate is where the savings are). Emit for each application the disposition, its priority, a written rationale in consultant language citing the specific scores, the pass/fail pattern and the evidence that drove the placement, plus a confidence level. The rationale, not the category, is the deliverable. [MVP] [Step 4 vocabulary settled 2026-08-13 by Bina: invest / consolidate / replace / retire, matching the hackathon prompt's own wording. The four terms are emitted directly, with no mapping to any other vocabulary - see the Notes sheet.]</t>
+          <t>(Step 4) Extend REQ 4: assign every application a disposition from exactly five categories - retain, invest, consolidate, replace, retire - using the pass/fail gate engine specified in REQ 52 rather than a business-value-by-technical-health 2x2 (a 2x2 has no axis on which 'consolidate' can appear, and consolidate is where the savings are). Emit for each application the disposition, its priority, a written rationale in consultant language citing the specific scores, the pass/fail pattern and the evidence that drove the placement, plus a confidence level. The rationale, not the category, is the deliverable. [MVP] [Step 4 vocabulary settled 2026-08-14 by Bina: retain / invest / consolidate / replace / retire. The five terms are emitted directly, with no mapping to any other vocabulary. Retain and invest are separate dispositions rather than one term read at two priorities: retain is a healthy application left alone with no new spend, invest is a funded remediation or enhancement - a deliberate injection of money or effort. This supersedes the four-term position of 2026-08-13, under which 'invest' carried both senses and only its priority told them apart - see the Notes sheet.]</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>(Steps 3-4) Implement disposition assignment as an explicit, configurable pass/fail lookup rather than a blended score. Gate each of the four scored dimensions - REQ 21 business value (V), REQ 22 technical health (T), REQ 23 cost efficiency (C), REQ 24 risk (R) - at a per-dimension threshold defaulting to 3.0 on the 1-5 scale, concatenate the four results into a VTCR key such as 'PPFP', and look that key up in an editable 16-row table returning one disposition from invest / consolidate / replace / retire and one priority from Very High / High / Moderate / Low / Very Low. Default table, to be argued with rather than assumed: PPPP invest (Very Low); PPPF invest (High); PPFP invest (Moderate); PPFF invest (High); PFPP invest (Moderate); PFPF invest (High); PFFP replace (High); PFFF replace (Very High); FPPP consolidate (Low); FPPF consolidate (Moderate); FPFP retire (High); FPFF retire (Very High); FFPP consolidate (Moderate); FFPF retire (High); FFFP retire (Very High); FFFF retire (Very High). Thresholds and every table row are configuration, not code. Score each criterion 1-5 in 0.5 increments with an integer weight per criterion where weight 0 disables it, and renormalise each dimension's weighted average over only the criteria that actually carry a value, so an application with sparse data is reported as incomplete by REQ 12 instead of being silently scored downward toward retire. Redundancy is not a gate: cluster membership from REQ 25 is an override that forces consolidate. REQ 51's lifecycle and sourcing exclusions run after the lookup. Store the VTCR key with the recommendation - it is the skeleton of REQ 27's rationale ('passes business value and cost efficiency, fails technical health and risk') - and allow the REQ 30 human override, validated against the same four-term vocabulary. [MVP] [REF: Infotech 04-Rationalize-Your-Application-Portfolio-Tool - weighted per-lens averages, 3.0 pass thresholds, four-character key and 16-row disposition truth table, disposition and priority held as separate fields; its blank-handling defect corrected here]</t>
+          <t>(Steps 3-4) Implement disposition assignment as an explicit, configurable pass/fail lookup rather than a blended score. Gate each of the four scored dimensions - REQ 21 business value (V), REQ 22 technical health (T), REQ 23 cost efficiency (C), REQ 24 risk (R) - at a per-dimension threshold defaulting to 3.0 on the 1-5 scale, concatenate the four results into a VTCR key such as 'PPFP', and look that key up in an editable 16-row table returning one disposition from retain / invest / consolidate / replace / retire and one priority from Very High / High / Moderate / Low / Very Low. Default table, to be argued with rather than assumed: PPPP retain (Very Low); PPPF invest (High); PPFP invest (Moderate); PPFF invest (High); PFPP invest (Moderate); PFPF invest (High); PFFP replace (High); PFFF replace (Very High); FPPP consolidate (Low); FPPF consolidate (Moderate); FPFP retire (High); FPFF retire (Very High); FFPP consolidate (Moderate); FFPF retire (High); FFFP retire (Very High); FFFF retire (Very High). The all-pass key PPPP is the only retain row, and it is what separates retain from invest: an application that clears every gate is healthy and needs no new spend, while every invest row fails at least one gate, so an invest recommendation always names the specific dimension the money is being spent on. Before 2026-08-14 PPPP returned invest at Very Low priority and those two cases were distinguished by priority alone; they are now distinct dispositions and priority is left to do only its own job. A failure of cost efficiency alone (PPFP) resolves to invest, never to retire. Thresholds and every table row are configuration, not code. Score each criterion 1-5 in 0.5 increments with an integer weight per criterion where weight 0 disables it, and renormalise each dimension's weighted average over only the criteria that actually carry a value, so an application with sparse data is reported as incomplete by REQ 12 instead of being silently scored downward toward retire. Redundancy is not a gate: cluster membership from REQ 25 is an override that forces consolidate. REQ 51's lifecycle and sourcing exclusions run after the lookup. Store the VTCR key with the recommendation - it is the skeleton of REQ 27's rationale ('passes business value and cost efficiency, fails technical health and risk') - and allow the REQ 30 human override, validated against the same five-term vocabulary. [MVP] [REF: Infotech 04-Rationalize-Your-Application-Portfolio-Tool - weighted per-lens averages, 3.0 pass thresholds, four-character key and 16-row disposition truth table, disposition and priority held as separate fields; its blank-handling defect corrected here]</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>(Steps 4-6) Separate recommendation from execution state as three distinct fields rather than overloading one: disposition (invest / consolidate / replace / retire), action (the specific verb - re-platform, upgrade, remediate, retrain, merge, absorb, decommission, modernize), and workflow status drawn from a controlled, configurable execution-stage vocabulary covering contract termination, compliance and archival review, application retirement, and per-team infrastructure decommission closure steps. Disposition answers what we recommend, action answers what will be done, status answers how far it has got - and status is what REQ 38's progress tracking reports against. [MVP for the three-field split and a first-pass status enum; STRETCH for the full multi-team execution pipeline] [REF: Infotech 04-Rationalize-Your-Application-Portfolio-Tool and 10-Disposition-Prioritization-Tool - both hold disposition and priority as separate fields; execution status has no equivalent in either and is defined by us]</t>
+          <t>(Steps 4-6) Separate recommendation from execution state as three distinct fields rather than overloading one: disposition (retain / invest / consolidate / replace / retire), action (the specific verb - monitor, re-platform, upgrade, remediate, retrain, merge, absorb, decommission, modernize), and workflow status drawn from a controlled, configurable execution-stage vocabulary covering contract termination, compliance and archival review, application retirement, and per-team infrastructure decommission closure steps. Disposition answers what we recommend, action answers what will be done, status answers how far it has got - and status is what REQ 38's progress tracking reports against. [MVP for the three-field split and a first-pass status enum; STRETCH for the full multi-team execution pipeline] [REF: Infotech 04-Rationalize-Your-Application-Portfolio-Tool and 10-Disposition-Prioritization-Tool - both hold disposition and priority as separate fields; execution status has no equivalent in either and is defined by us]</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Ryo's Sheet1 columns (Requirement ID / Category / AI Tool Requirement Description) are unchanged, and requirements 1-5 are exactly as he wrote them. New rows continue his numbering from 6, now running to 65. Nothing was renamed, reordered, or overwritten; where an existing added requirement needed correcting (10, 16, 19, 20, 21, 22, 23, 24, 25, 27, 29, 32) it was edited in place and the change is recorded below.</t>
+          <t>Ryo's Sheet1 columns (Requirement ID / Category / AI Tool Requirement Description) are unchanged, and requirements 1-5 are exactly as he wrote them apart from REQ 4, where the five-term disposition vocabulary decided on 2026-08-14 was corrected in place (vocabulary only, no change of meaning) - the single edit to his rows. New rows continue his numbering from 6, now running to 65. Nothing was renamed, reordered, or overwritten; where an existing added requirement needed correcting (10, 16, 19, 20, 21, 22, 23, 24, 25, 27, 29, 32) it was edited in place and the change is recorded below. The 2026-08-14 vocabulary change edited 4, 27, 52 and 64 in place; the requirement count stays at 65 and nothing was split.</t>
         </is>
       </c>
     </row>
@@ -1585,6 +1585,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
@@ -1701,6 +1702,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -1712,150 +1714,199 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Step 4 vocabulary - DECIDED 2026-08-13</t>
+          <t>Step 4 vocabulary - DECIDED 2026-08-14 (supersedes 2026-08-13)</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>DECIDED by Bina on 2026-08-13 at 4:23pm ET: the disposition vocabulary is exactly four terms - invest, consolidate, replace, retire - chosen to match the wording of the hackathon prompt itself, which is also what Ryo's REQ 4 already said. The engine emits those four directly. There is no mapping layer to slide 13's retain / replace / retire and no five-category variant with a separate 'retain'; the earlier recommendation to map down to slide 13's three terms is withdrawn. One supporting observation worth keeping: every Info-Tech tool we reviewed keeps a consolidate-equivalent (Consolidate, Merge, Absorb, Refocus) while slide 13 does not, which supports the choice - consolidation is where the savings story lives (REQ 25). One consequence to build to: with no separate 'retain' term, 'invest' covers both a healthy application kept as it is and one carrying a funded remediation; the two are distinguished by the REQ 52 pass/fail pattern and priority, which are stored with every disposition. Requirements carrying this decision: 4 (Ryo's, already consistent), 27, 52, 64.</t>
+          <t>DECIDED by Bina Din on 2026-08-14: the disposition vocabulary is five terms - retain, invest, consolidate, replace, retire. Asked to confirm that the four-term version read correctly in front of a steering committee, her answer was: 'No, separate by invest, retain, consolidate, replace, and retire.' Definitions, to be used exactly as written in every output: RETAIN - healthy, leave alone, no new spend. INVEST - fund a remediation or enhancement; a deliberate injection of money or effort. CONSOLIDATE - fold into another application that covers the same capability. REPLACE - swap for a different product. RETIRE - decommission. This SUPERSEDES the four-term position decided on 2026-08-13 (invest, consolidate, replace, retire, chosen to match the wording of the hackathon prompt itself and of Ryo's REQ 4), under which 'invest' did double duty for both a healthy application kept as it is and one carrying a funded remediation, the two separated only by priority and the REQ 52 pass/fail pattern. That separation was legible inside the engine and not on the page: a steering-committee reader cannot be expected to infer which sense of 'invest' is meant from a priority value, and 'invest' against a healthy application reads as a request for money that nobody is asking for. The engine emits the five terms directly; there is still no mapping layer to any other vocabulary, and slide 13's retain / replace / retire remains a subset of ours rather than a target to map down to. Mechanically the change is small and contained in REQ 52's lookup table: the all-pass key PPPP, previously invest at Very Low priority, now returns retain, and every remaining invest row fails at least one gate, so invest always names the dimension it is funding. The supporting observation from 2026-08-13 still holds - every Info-Tech tool reviewed keeps a consolidate-equivalent (Consolidate, Merge, Absorb, Refocus) while slide 13 does not, and consolidation is where the savings story lives (REQ 25). Requirements carrying this decision: 4 (Ryo's, edited for vocabulary only), 27, 52, 64.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Synthetic data scope</t>
+          <t>Risk in the scoring engine - DECIDED 2026-08-14</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>The overarching prompt describes a 600-application portfolio, so the demo runs on a synthetic portfolio generated to that scale. No client operational data is ingested, used, or committed (see 'Client data - out of scope' below). What must be synthesized, by field category: business-capability tags (REQ 19); active-usage telemetry as distinct from purchased entitlements (REQ 21, 23); most of the per-component TCO breakdown (REQ 20, 55); risk attributes, technical, compliance and clinical (REQ 24, 65); dependency edges and the infrastructure/data footprint (REQ 10, 57); lifecycle stage and sourcing type (REQ 51); retention and archival obligations (REQ 53); and contract terms beyond identifier and end date (REQ 16). Generation rules must be published alongside the data so nothing modelled can be mistaken for measured (REQ 49). Still needs a yes on scale and generation approach before the scoring work starts - it remains the biggest single scope dependency on the sheet.</t>
+          <t>DECIDED by Bina Din on 2026-08-14: risk stays substituted into the borrowed engine's end-user dimension slot. The Info-Tech portfolio tool that REQ 52 borrows its mechanism from scores end-user perception as its fourth dimension; we score risk there instead - REQ 24's technical and business/compliance axes plus REQ 65's clinical and patient-safety axis - so the R in the VTCR key is risk, and a risk failure is a gate failure rather than a footnote. End-user perception is still collected as a field, at integer weight 0, which under REQ 52's renormalisation means it is recorded and reported but never moves a score; a client who wants it scored raises the weight rather than waiting for a rebuild. In a health system an application nobody likes is a training problem, while an application holding PHI on an unpatched host is a board-level one, and only one of those belongs in a gate.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Capability taxonomy</t>
+          <t>Cost in the disposition - DECIDED 2026-08-14</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Requirement 19 assumes we adopt an existing published health-system business capability model rather than authoring one on build day. Bina to confirm which one, since every redundancy finding depends on it.</t>
+          <t>DECIDED by Bina Din on 2026-08-14: cost moves priority, but cost can never on its own make something a retire. Cost efficiency (REQ 23) stays a scored gate and remains a first-order driver of priority and of wave sequencing (REQ 31, REQ 56), so an expensive application surfaces early and loudly. But a cost failure with business value, technical health and risk all passing - the PPFP row of REQ 52's table - resolves to invest, not retire, and no row where cost is the only failure may ever be mapped to retire. An application is retired for lack of value, for being unsupportable, or for carrying unacceptable risk; being expensive makes a decision urgent, not inevitable. Anyone editing the 16-row table has to preserve this.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Demo scope</t>
+          <t>Value dimension weighting - DECIDED 2026-08-14</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Steps 6 and 7 (requirements 37-45) describe post-decision capability, which normally implies a real program running over months. Two of them are demoable on Friday without that: 38 (progress tracking) and 41 (realized vs projected savings) both work by feeding the tool two snapshots of the same portfolio. Worth deciding whether to build one of those, because a tool that closes the loop on whether the savings actually landed is a materially stronger pitch than one that stops at the recommendation.</t>
+          <t>DECIDED by Bina Din on 2026-08-14: inside REQ 21's business value dimension, criticality to patient care takes the double weight (integer weight 2 in REQ 52's per-criterion weighting), and governance and compliance drop to weight 1. Patient-care criticality is the first criterion a clinical stakeholder tests the model against, and it should outweigh a governance attribute rather than sit level with it. Note this is the value dimension only - compliance exposure is still scored at full strength as risk in REQ 24, so lowering its weight here de-duplicates it rather than discounting it, consistent with the one-signal-one-dimension partition below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Cost efficiency benchmark - DECIDED 2026-08-14</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>DECIDED by Bina Din on 2026-08-14: REQ 23's cost efficiency continues to use the modelled peer band - cost per active user compared against the band formed by the other applications carrying the same business capability tag inside the portfolio. That band is modelled, not measured against any external benchmark, published market rate or industry dataset, and every output that uses it must say so under REQ 49's no-silent-inference rule, so a within-portfolio comparison is never read as an industry benchmark. It is a defensible relative signal and an indefensible absolute one, and the outputs have to state which of the two they are.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Reference material</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n"/>
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Synthetic data scope</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>The overarching prompt describes a 600-application portfolio, so the demo runs on a synthetic portfolio generated to that scale. No client operational data is ingested, used, or committed (see 'Client data - out of scope' below). What must be synthesized, by field category: business-capability tags (REQ 19); active-usage telemetry as distinct from purchased entitlements (REQ 21, 23); most of the per-component TCO breakdown (REQ 20, 55); risk attributes, technical, compliance and clinical (REQ 24, 65); dependency edges and the infrastructure/data footprint (REQ 10, 57); lifecycle stage and sourcing type (REQ 51); retention and archival obligations (REQ 53); and contract terms beyond identifier and end date (REQ 16). Generation rules must be published alongside the data so nothing modelled can be mistaken for measured (REQ 49). Still needs a yes on scale and generation approach before the scoring work starts - it remains the biggest single scope dependency on the sheet.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Slide 13 - READ and incorporated</t>
+          <t>Capability taxonomy</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>The seven-step process from slide 13 of Bina's Novant playbook is now the organizing spine of this sheet; every added requirement carries a (Step N) marker and the coverage map above is built from it. Source: the slide-13 image Ryo posted in #hack-team-12 on 2026-08-12, immediately after suggesting we hang AI insertion points off that workflow.</t>
+          <t>Requirement 19 assumes we adopt an existing published health-system business capability model rather than authoring one on build day. Bina to confirm which one, since every redundancy finding depends on it.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Infotech templates - READ 2026-08-13</t>
+          <t>Demo scope</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>All five Info-Tech references Bina shared were read in full on 2026-08-13 (02-Application-Portfolio-Management-Diagnostic-Tool, 02-Build-an-Application-Rationalization-Framework, 04-Rationalize-Your-Application-Portfolio-Tool, 05-Application-TCO-Calculator, 10-Disposition-Prioritization-Tool), which replaces the earlier 'not read' caveat on this row. What they validated: the scoring dimensions behind REQ 21-24 (weighted multi-lens scoring, gates, then disposition plus priority, is still current practice and matches what Gartner TIME, LeanIX, Apptio and ServiceNow APM do today); the TCO component taxonomy now enumerated in REQ 20 and REQ 55; the prioritisation axes in REQ 56; and the disposition mechanism now specified in REQ 52, which is borrowed from the portfolio tool rather than invented. Two genuine obsolescence findings, both of which we have to fix rather than copy: (1) there is no line item anywhere in the reference cost model for consumption or usage-based pricing, which is now the dominant SaaS metric and the primary cost model for the AI tools the prompt calls out - REQ 20 and REQ 55 add it with no precedent to borrow; (2) every scoring input in every template assumes a human fills in a 1-5 grid in a facilitated workshop, which is precisely the step this agent removes - the methodology is current, its data acquisition is a decade behind, and that gap is the pitch (REQ 6-8 derive usage, spend and shadow IT from SSO, AP and contract data instead of asking people). Build caution: the files are internally inconsistent in places - duplicated and misspelled subtotal labels, dropdown lists feeding columns they no longer match, named ranges resolving to #REF!, and one disposition category defined but unreachable from its own lookup table - so nothing was ported without checking it against the file's own cached values, and anything not already written into these requirements should be re-derived rather than copied. Scale note: those tools cap at roughly 500, 25 and 12 records respectively, so they are unusable as tools at 600 applications - only their logic ports. They are licensed third-party vendor material and this repo is public: cite them, never reproduce or commit them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>AI requirements - no external validation</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>None of the reference material mentions AI at all - zero occurrences across all five Info-Tech templates and slide 13's seven-step process. REQ 11 (AI tools and agents as a first-class inventory category), REQ 26 (a capability bought standalone that is already entitled inside an existing enterprise licence) and the consumption-pricing component in REQ 20 and REQ 55 therefore have no external cross-check available: no precedent, no field taxonomy, no scoring rubric. That makes them simultaneously the clearest differentiator on this sheet and the part with the least outside validation, so they need the most internal scrutiny before Friday - someone other than the author should review those requirements specifically.</t>
-        </is>
-      </c>
-    </row>
+          <t>Steps 6 and 7 (requirements 37-45) describe post-decision capability, which normally implies a real program running over months. Two of them are demoable on Friday without that: 38 (progress tracking) and 41 (realized vs projected savings) both work by feeding the tool two snapshots of the same portfolio. Worth deciding whether to build one of those, because a tool that closes the loop on whether the savings actually landed is a materially stronger pitch than one that stops at the recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Dependency guardrail - DECIDED</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>The sheet previously tagged REQ 10 (dependency map) and REQ 29 (breakage and renewal test) STRETCH while REQ 25 (consolidation recommendations) and REQ 27 (disposition assignment) were MVP - so as specified, the Friday tool would recommend retirements and consolidations with no breakage check at all. Of the two available fixes, promote the guardrail or scope consolidation MVP to explicitly disclaim breakage safety, we chose to PROMOTE. REQ 10 now ships an MVP minimum: a per-application has_downstream_dependents boolean plus an enabling / dependent / overlapping flag on each application pair, which is three letters per cell and no formulas. REQ 29's minimum check against that signal, the renewal calendar and REQ 53's retention expiry is MVP too, and REQ 25 now states that every cluster recommendation is checked before it is published. The full confidence-weighted edge list and edge-level deferral scheduling stay STRETCH.</t>
-        </is>
-      </c>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Reference material</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Cost and savings model - corrected</t>
+          <t>Slide 13 - READ and incorporated</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Two arithmetic corrections, both of which move the headline number. (1) REQ 20's component list went from four components to eight: licence and subscription; external support and maintenance; version-upgrade and additional-module fees; internal labour; infrastructure; indirect and training costs; consumption / usage-based charges; and one-time implementation cost held separately from the recurring run-rate. Upgrade and module fees, indirect and training cost, and one-time implementation were all missing, and under-counted cost under-counts savings against the 15% target. REQ 55 carries the published estimation rule for every modelled component. (2) REQ 32 now computes net rather than gross saving - current TCO, minus the replacement or survivor's ongoing TCO, minus amortised one-time migration and implementation cost, minus residual archival and retention cost where a REQ 53 obligation outlives the application - and REQ 54 requires every figure reported both as an annual run-rate and as an undiscounted five-year cumulative. A retire recommendation does not return 100% of an application's cost; in a regulated environment retire is both the disposition most likely to be blocked and the one most likely to leave residual cost behind.</t>
+          <t>The seven-step process from slide 13 of Bina's Novant playbook is now the organizing spine of this sheet; every added requirement carries a (Step N) marker and the coverage map above is built from it. Source: the slide-13 image Ryo posted in #hack-team-12 on 2026-08-12, immediately after suggesting we hang AI insertion points off that workflow.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Scoring input partition</t>
+          <t>Infotech templates - READ 2026-08-13</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Business value (REQ 21), technical health (REQ 22), cost efficiency (REQ 23) and risk (REQ 24) previously shared inputs: unsupported versions and vendor viability were scored in both technical health and risk, so one obsolescence fact failed two of the four gates and the engine systematically over-recommended retiring old-but-adequate applications. Every signal now belongs to exactly one dimension, stated in the text of each requirement so the partition survives into the build. REQ 22 owns version currency, EOL proximity, unsupported-version status, architecture fit, operational stability and vendor viability. REQ 24 owns single points of failure, absent DR or backup, single-vendor concentration, unhardened configuration, PHI and HIPAA exposure, data residency, SOC 2 / HITRUST posture and contractual lock-in. REQ 65 owns the clinical and patient-safety axis. REQ 23 owns the cost signals. REQ 21 owns criticality, usage breadth, process centrality and owner-stated strategic importance.</t>
+          <t>All five Info-Tech references Bina shared were read in full on 2026-08-13 (02-Application-Portfolio-Management-Diagnostic-Tool, 02-Build-an-Application-Rationalization-Framework, 04-Rationalize-Your-Application-Portfolio-Tool, 05-Application-TCO-Calculator, 10-Disposition-Prioritization-Tool), which replaces the earlier 'not read' caveat on this row. What they validated: the scoring dimensions behind REQ 21-24 (weighted multi-lens scoring, gates, then disposition plus priority, is still current practice and matches what Gartner TIME, LeanIX, Apptio and ServiceNow APM do today); the TCO component taxonomy now enumerated in REQ 20 and REQ 55; the prioritisation axes in REQ 56; and the disposition mechanism now specified in REQ 52, which is borrowed from the portfolio tool rather than invented. Two genuine obsolescence findings, both of which we have to fix rather than copy: (1) there is no line item anywhere in the reference cost model for consumption or usage-based pricing, which is now the dominant SaaS metric and the primary cost model for the AI tools the prompt calls out - REQ 20 and REQ 55 add it with no precedent to borrow; (2) every scoring input in every template assumes a human fills in a 1-5 grid in a facilitated workshop, which is precisely the step this agent removes - the methodology is current, its data acquisition is a decade behind, and that gap is the pitch (REQ 6-8 derive usage, spend and shadow IT from SSO, AP and contract data instead of asking people). Build caution: the files are internally inconsistent in places - duplicated and misspelled subtotal labels, dropdown lists feeding columns they no longer match, named ranges resolving to #REF!, and one disposition category defined but unreachable from its own lookup table - so nothing was ported without checking it against the file's own cached values, and anything not already written into these requirements should be re-derived rather than copied. Scale note: those tools cap at roughly 500, 25 and 12 records respectively, so they are unusable as tools at 600 applications - only their logic ports. They are licensed third-party vendor material and this repo is public: cite them, never reproduce or commit them.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Disposition engine - specified</t>
+          <t>AI requirements - no external validation</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>REQ 52 pins the mechanism the sheet previously left open, concretely enough to code: gate REQ 21, 22, 23 and 24 at 3.0 on the 1-5 scale, concatenate the four pass/fail results into a VTCR key, look that key up in a 16-row editable table returning one of the four agreed dispositions plus a priority (Very High through Very Low), store the key as the human-readable rationale skeleton REQ 27 needs, force consolidate wherever REQ 25 finds cluster membership, apply REQ 51's lifecycle and sourcing exclusions after the lookup and record every suppression with its reason, and allow the REQ 30 human override validated against the same four terms. The default 16-row mapping is written into REQ 52 and is configuration rather than code, which means a client can argue with the table directly instead of with a black box. Note also that the value-by-health 2x2 in REQ 4 and REQ 27 remains the right chart but cannot be the engine: a 2x2 has no axis on which 'consolidate' can appear, and consolidate is where the savings are.</t>
+          <t>None of the reference material mentions AI at all - zero occurrences across all five Info-Tech templates and slide 13's seven-step process. REQ 11 (AI tools and agents as a first-class inventory category), REQ 26 (a capability bought standalone that is already entitled inside an existing enterprise licence) and the consumption-pricing component in REQ 20 and REQ 55 therefore have no external cross-check available: no precedent, no field taxonomy, no scoring rubric. That makes them simultaneously the clearest differentiator on this sheet and the part with the least outside validation, so they need the most internal scrutiny before Friday - someone other than the author should review those requirements specifically.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
+          <t>Dependency guardrail - DECIDED</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>The sheet previously tagged REQ 10 (dependency map) and REQ 29 (breakage and renewal test) STRETCH while REQ 25 (consolidation recommendations) and REQ 27 (disposition assignment) were MVP - so as specified, the Friday tool would recommend retirements and consolidations with no breakage check at all. Of the two available fixes, promote the guardrail or scope consolidation MVP to explicitly disclaim breakage safety, we chose to PROMOTE. REQ 10 now ships an MVP minimum: a per-application has_downstream_dependents boolean plus an enabling / dependent / overlapping flag on each application pair, which is three letters per cell and no formulas. REQ 29's minimum check against that signal, the renewal calendar and REQ 53's retention expiry is MVP too, and REQ 25 now states that every cluster recommendation is checked before it is published. The full confidence-weighted edge list and edge-level deferral scheduling stay STRETCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Cost and savings model - corrected</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Two arithmetic corrections, both of which move the headline number. (1) REQ 20's component list went from four components to eight: licence and subscription; external support and maintenance; version-upgrade and additional-module fees; internal labour; infrastructure; indirect and training costs; consumption / usage-based charges; and one-time implementation cost held separately from the recurring run-rate. Upgrade and module fees, indirect and training cost, and one-time implementation were all missing, and under-counted cost under-counts savings against the 15% target. REQ 55 carries the published estimation rule for every modelled component. (2) REQ 32 now computes net rather than gross saving - current TCO, minus the replacement or survivor's ongoing TCO, minus amortised one-time migration and implementation cost, minus residual archival and retention cost where a REQ 53 obligation outlives the application - and REQ 54 requires every figure reported both as an annual run-rate and as an undiscounted five-year cumulative. A retire recommendation does not return 100% of an application's cost; in a regulated environment retire is both the disposition most likely to be blocked and the one most likely to leave residual cost behind.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Scoring input partition</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Business value (REQ 21), technical health (REQ 22), cost efficiency (REQ 23) and risk (REQ 24) previously shared inputs: unsupported versions and vendor viability were scored in both technical health and risk, so one obsolescence fact failed two of the four gates and the engine systematically over-recommended retiring old-but-adequate applications. Every signal now belongs to exactly one dimension, stated in the text of each requirement so the partition survives into the build. REQ 22 owns version currency, EOL proximity, unsupported-version status, architecture fit, operational stability and vendor viability. REQ 24 owns single points of failure, absent DR or backup, single-vendor concentration, unhardened configuration, PHI and HIPAA exposure, data residency, SOC 2 / HITRUST posture and contractual lock-in. REQ 65 owns the clinical and patient-safety axis. REQ 23 owns the cost signals. REQ 21 owns criticality, usage breadth, process centrality and owner-stated strategic importance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Disposition engine - specified</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>REQ 52 pins the mechanism the sheet previously left open, concretely enough to code: gate REQ 21, 22, 23 and 24 at 3.0 on the 1-5 scale, concatenate the four pass/fail results into a VTCR key, look that key up in a 16-row editable table returning one of the five agreed dispositions plus a priority (Very High through Very Low), the all-pass key PPPP returning retain since 2026-08-14 while every invest row fails at least one gate, store the key as the human-readable rationale skeleton REQ 27 needs, force consolidate wherever REQ 25 finds cluster membership, apply REQ 51's lifecycle and sourcing exclusions after the lookup and record every suppression with its reason, and allow the REQ 30 human override validated against the same five terms. The default 16-row mapping is written into REQ 52 and is configuration rather than code, which means a client can argue with the table directly instead of with a black box. Note also that the value-by-health 2x2 in REQ 4 and REQ 27 remains the right chart but cannot be the engine: a 2x2 has no axis on which 'consolidate' can appear, and consolidate is where the savings are.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
           <t>Client data - out of scope</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Bina ruled client operational data out of scope on 2026-08-13. Nothing in this workbook derives from it: no application inventory, no named individuals, no contract identifiers, no cost or contract actuals, no server names, and no departments or legal entities appear anywhere in these requirements, and none may be added. This repository is public, which means there is no access-control boundary of any kind and git history is permanent, so the same standard applies to every file committed here - generic methodology and field names are in scope, client content is not. The demo runs on the synthetic portfolio described above.</t>
         </is>

</xml_diff>